<commit_message>
Client and LCSC BOM updated issue #28
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/Client-BOM_Bottom_PCB.xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/Client-BOM_Bottom_PCB.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9904CAF1-D14C-4FA0-B9DB-ED4CEDE5700C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="10335" windowHeight="10620"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SM_Bottom_Board" sheetId="1" r:id="rId1"/>
@@ -17,17 +18,24 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">SM_Bottom_Board!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="214">
   <si>
     <t>Description</t>
   </si>
@@ -669,12 +677,15 @@
   </si>
   <si>
     <t xml:space="preserve"> Link</t>
+  </si>
+  <si>
+    <t>Custom Supplier</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.000"/>
@@ -1235,7 +1246,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1518,13 +1529,16 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1548,13 +1562,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1837,7 +1851,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1857,7 +1871,7 @@
     <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" customWidth="1"/>
     <col min="15" max="15" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21.85546875" bestFit="1" customWidth="1"/>
@@ -1866,27 +1880,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="107" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="97"/>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="97"/>
-      <c r="K1" s="97"/>
-      <c r="L1" s="97"/>
-      <c r="M1" s="97"/>
-      <c r="N1" s="97"/>
-      <c r="O1" s="97"/>
-      <c r="P1" s="97"/>
-      <c r="Q1" s="97"/>
-      <c r="R1" s="97"/>
-      <c r="S1" s="98"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="108"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="108"/>
+      <c r="O1" s="108"/>
+      <c r="P1" s="108"/>
+      <c r="Q1" s="108"/>
+      <c r="R1" s="108"/>
+      <c r="S1" s="109"/>
     </row>
     <row r="2" spans="1:19" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="28" t="s">
@@ -1951,7 +1965,7 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="99" t="s">
+      <c r="B3" s="100" t="s">
         <v>144</v>
       </c>
       <c r="C3" s="65" t="s">
@@ -2011,7 +2025,7 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="100"/>
+      <c r="B4" s="101"/>
       <c r="C4" s="66" t="s">
         <v>179</v>
       </c>
@@ -2069,7 +2083,7 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="100"/>
+      <c r="B5" s="101"/>
       <c r="C5" s="66" t="s">
         <v>13</v>
       </c>
@@ -2127,7 +2141,7 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="100"/>
+      <c r="B6" s="101"/>
       <c r="C6" s="66" t="s">
         <v>18</v>
       </c>
@@ -2185,7 +2199,7 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="100"/>
+      <c r="B7" s="101"/>
       <c r="C7" s="66" t="s">
         <v>24</v>
       </c>
@@ -2243,7 +2257,7 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="101"/>
+      <c r="B8" s="102"/>
       <c r="C8" s="67" t="s">
         <v>30</v>
       </c>
@@ -2301,7 +2315,7 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="99" t="s">
+      <c r="B9" s="100" t="s">
         <v>145</v>
       </c>
       <c r="C9" s="65" t="s">
@@ -2363,7 +2377,7 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="100"/>
+      <c r="B10" s="101"/>
       <c r="C10" s="66" t="s">
         <v>39</v>
       </c>
@@ -2421,7 +2435,7 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="101"/>
+      <c r="B11" s="102"/>
       <c r="C11" s="67" t="s">
         <v>52</v>
       </c>
@@ -2597,7 +2611,7 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="99" t="s">
+      <c r="B14" s="100" t="s">
         <v>147</v>
       </c>
       <c r="C14" s="65" t="s">
@@ -2657,7 +2671,7 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="100"/>
+      <c r="B15" s="101"/>
       <c r="C15" s="66" t="s">
         <v>72</v>
       </c>
@@ -2715,7 +2729,7 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="100"/>
+      <c r="B16" s="101"/>
       <c r="C16" s="66" t="s">
         <v>195</v>
       </c>
@@ -2773,7 +2787,7 @@
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="100"/>
+      <c r="B17" s="101"/>
       <c r="C17" s="66" t="s">
         <v>80</v>
       </c>
@@ -2831,7 +2845,7 @@
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="100"/>
+      <c r="B18" s="101"/>
       <c r="C18" s="66" t="s">
         <v>84</v>
       </c>
@@ -2889,7 +2903,7 @@
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="101"/>
+      <c r="B19" s="102"/>
       <c r="C19" s="67" t="s">
         <v>174</v>
       </c>
@@ -3007,7 +3021,7 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="99" t="s">
+      <c r="B21" s="100" t="s">
         <v>149</v>
       </c>
       <c r="C21" s="65" t="s">
@@ -3067,7 +3081,7 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="101"/>
+      <c r="B22" s="102"/>
       <c r="C22" s="67" t="s">
         <v>131</v>
       </c>
@@ -3123,7 +3137,7 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="99" t="s">
+      <c r="B23" s="100" t="s">
         <v>150</v>
       </c>
       <c r="C23" s="79" t="s">
@@ -3183,7 +3197,7 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="100"/>
+      <c r="B24" s="101"/>
       <c r="C24" s="87" t="s">
         <v>98</v>
       </c>
@@ -3199,10 +3213,18 @@
       <c r="G24" s="88" t="s">
         <v>101</v>
       </c>
-      <c r="H24" s="89"/>
-      <c r="I24" s="89"/>
-      <c r="J24" s="88"/>
-      <c r="K24" s="88"/>
+      <c r="H24" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="I24" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="J24" s="88" t="s">
+        <v>196</v>
+      </c>
+      <c r="K24" s="89">
+        <v>25</v>
+      </c>
       <c r="L24" s="89">
         <v>1</v>
       </c>
@@ -3210,16 +3232,22 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="N24" s="90"/>
-      <c r="O24" s="91"/>
+      <c r="N24" s="90" t="s">
+        <v>213</v>
+      </c>
+      <c r="O24" s="91">
+        <v>13.69</v>
+      </c>
       <c r="P24" s="91">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="Q24" s="91"/>
+        <v>13.69</v>
+      </c>
+      <c r="Q24" s="91">
+        <v>13.69</v>
+      </c>
       <c r="R24" s="91">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>342.25</v>
       </c>
       <c r="S24" s="92"/>
     </row>
@@ -3227,7 +3255,7 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="100"/>
+      <c r="B25" s="101"/>
       <c r="C25" s="66" t="s">
         <v>103</v>
       </c>
@@ -3285,7 +3313,7 @@
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="100"/>
+      <c r="B26" s="101"/>
       <c r="C26" s="66" t="s">
         <v>108</v>
       </c>
@@ -3343,7 +3371,7 @@
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="100"/>
+      <c r="B27" s="101"/>
       <c r="C27" s="66" t="s">
         <v>113</v>
       </c>
@@ -3401,7 +3429,7 @@
       <c r="A28" s="1">
         <v>26</v>
       </c>
-      <c r="B28" s="100"/>
+      <c r="B28" s="101"/>
       <c r="C28" s="66" t="s">
         <v>117</v>
       </c>
@@ -3459,7 +3487,7 @@
       <c r="A29" s="1">
         <v>27</v>
       </c>
-      <c r="B29" s="101"/>
+      <c r="B29" s="102"/>
       <c r="C29" s="67" t="s">
         <v>122</v>
       </c>
@@ -3517,7 +3545,7 @@
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" s="104" t="s">
+      <c r="B30" s="105" t="s">
         <v>151</v>
       </c>
       <c r="C30" s="70" t="s">
@@ -3577,7 +3605,7 @@
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="104"/>
+      <c r="B31" s="105"/>
       <c r="C31" s="87" t="s">
         <v>44</v>
       </c>
@@ -3593,10 +3621,18 @@
       <c r="G31" s="88" t="s">
         <v>46</v>
       </c>
-      <c r="H31" s="89"/>
-      <c r="I31" s="89"/>
-      <c r="J31" s="88"/>
-      <c r="K31" s="88"/>
+      <c r="H31" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="I31" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="J31" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="K31" s="89">
+        <v>30</v>
+      </c>
       <c r="L31" s="89">
         <v>1</v>
       </c>
@@ -3604,16 +3640,22 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="N31" s="90"/>
-      <c r="O31" s="93"/>
+      <c r="N31" s="90" t="s">
+        <v>213</v>
+      </c>
+      <c r="O31" s="93">
+        <v>2.56</v>
+      </c>
       <c r="P31" s="91">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="Q31" s="93"/>
+        <v>2.56</v>
+      </c>
+      <c r="Q31" s="93">
+        <v>2.56</v>
+      </c>
       <c r="R31" s="91">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>76.8</v>
       </c>
       <c r="S31" s="92"/>
     </row>
@@ -3621,7 +3663,7 @@
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="104"/>
+      <c r="B32" s="105"/>
       <c r="C32" s="87" t="s">
         <v>57</v>
       </c>
@@ -3637,10 +3679,18 @@
       <c r="G32" s="88" t="s">
         <v>59</v>
       </c>
-      <c r="H32" s="89"/>
-      <c r="I32" s="89"/>
-      <c r="J32" s="88"/>
-      <c r="K32" s="88"/>
+      <c r="H32" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="I32" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="J32" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="K32" s="89">
+        <v>30</v>
+      </c>
       <c r="L32" s="89">
         <v>1</v>
       </c>
@@ -3648,16 +3698,22 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="N32" s="90"/>
-      <c r="O32" s="89"/>
+      <c r="N32" s="90" t="s">
+        <v>213</v>
+      </c>
+      <c r="O32" s="99">
+        <v>0.5</v>
+      </c>
       <c r="P32" s="91">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="Q32" s="91"/>
+        <v>0.5</v>
+      </c>
+      <c r="Q32" s="99">
+        <v>0.5</v>
+      </c>
       <c r="R32" s="91">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="S32" s="92"/>
     </row>
@@ -3665,7 +3721,7 @@
       <c r="A33" s="74">
         <v>31</v>
       </c>
-      <c r="B33" s="105"/>
+      <c r="B33" s="106"/>
       <c r="C33" s="75" t="s">
         <v>205</v>
       </c>
@@ -3694,51 +3750,51 @@
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="N33" s="106" t="s">
+      <c r="N33" s="96" t="s">
         <v>196</v>
       </c>
-      <c r="O33" s="106" t="s">
+      <c r="O33" s="96" t="s">
         <v>196</v>
       </c>
-      <c r="P33" s="107" t="s">
+      <c r="P33" s="97" t="s">
         <v>181</v>
       </c>
-      <c r="Q33" s="106" t="s">
+      <c r="Q33" s="96" t="s">
         <v>196</v>
       </c>
-      <c r="R33" s="106" t="s">
+      <c r="R33" s="96" t="s">
         <v>196</v>
       </c>
-      <c r="S33" s="108" t="s">
+      <c r="S33" s="98" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="L34" s="102" t="s">
+      <c r="L34" s="103" t="s">
         <v>153</v>
       </c>
-      <c r="M34" s="102"/>
-      <c r="N34" s="102"/>
-      <c r="O34" s="102"/>
+      <c r="M34" s="103"/>
+      <c r="N34" s="103"/>
+      <c r="O34" s="103"/>
       <c r="R34" s="3">
         <f>SUM(R3:R33)</f>
-        <v>822.35699999999997</v>
+        <v>1256.4069999999999</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="L35" s="103" t="s">
+      <c r="L35" s="104" t="s">
         <v>154</v>
       </c>
-      <c r="M35" s="103"/>
-      <c r="N35" s="103"/>
-      <c r="O35" s="103"/>
+      <c r="M35" s="104"/>
+      <c r="N35" s="104"/>
+      <c r="O35" s="104"/>
       <c r="P35" s="2">
         <f>SUM(P3:P34)</f>
-        <v>86.865479999999991</v>
+        <v>103.61547999999999</v>
       </c>
       <c r="R35" s="4">
         <f>R34/25</f>
-        <v>32.894280000000002</v>
+        <v>50.256279999999997</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
@@ -3843,33 +3899,33 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N3" r:id="rId1"/>
-    <hyperlink ref="N4" r:id="rId2"/>
-    <hyperlink ref="N7" r:id="rId3"/>
-    <hyperlink ref="N8" r:id="rId4"/>
-    <hyperlink ref="N11" r:id="rId5"/>
-    <hyperlink ref="N14" r:id="rId6"/>
-    <hyperlink ref="N15" r:id="rId7"/>
-    <hyperlink ref="N16" r:id="rId8"/>
-    <hyperlink ref="N17" r:id="rId9"/>
-    <hyperlink ref="N18" r:id="rId10"/>
-    <hyperlink ref="N19" r:id="rId11"/>
-    <hyperlink ref="N27" r:id="rId12"/>
-    <hyperlink ref="N29" r:id="rId13"/>
-    <hyperlink ref="N28" r:id="rId14"/>
-    <hyperlink ref="N26" r:id="rId15"/>
-    <hyperlink ref="N25" r:id="rId16"/>
-    <hyperlink ref="N6" r:id="rId17"/>
-    <hyperlink ref="N9" r:id="rId18"/>
-    <hyperlink ref="N10" r:id="rId19"/>
-    <hyperlink ref="N12" r:id="rId20"/>
-    <hyperlink ref="N13" r:id="rId21"/>
-    <hyperlink ref="N20" r:id="rId22"/>
-    <hyperlink ref="N22" r:id="rId23"/>
-    <hyperlink ref="N23" r:id="rId24"/>
-    <hyperlink ref="N30" r:id="rId25"/>
-    <hyperlink ref="N5" r:id="rId26"/>
-    <hyperlink ref="N21" r:id="rId27"/>
+    <hyperlink ref="N3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N11" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N14" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N15" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N16" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N17" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N18" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N19" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N27" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N29" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="N28" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="N26" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="N25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="N6" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="N9" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="N10" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="N12" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N13" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="N20" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="N22" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="N23" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="N30" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N5" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="N21" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>

</xml_diff>